<commit_message>
app furtinure finish 20260815
</commit_message>
<xml_diff>
--- a/PROYECTOS/MEZANINE MA/Lista de materiales.xlsx
+++ b/PROYECTOS/MEZANINE MA/Lista de materiales.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30330"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30411"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VIC\Downloads\CURSO SKETCHUP\PROYECTOS\MEZANINE MA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3489AF33-2659-4FD6-BC2F-B87FE8F0B7A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6B61417-D371-4BB9-9BE7-07FF4E4F20E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{9C38CAA7-9F0A-40CC-8992-24B3D9ED1EBA}"/>
   </bookViews>
@@ -18,6 +18,7 @@
     <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="190">
   <si>
     <t>LISTA DE MATERIALES</t>
   </si>
@@ -445,12 +446,6 @@
     <t>100 Tornillos 3.5x15mm (melamina 15mm, bisagras y correderas)</t>
   </si>
   <si>
-    <t>100 Tornillos 4.0x50mm (melamina 15mm)</t>
-  </si>
-  <si>
-    <t>100 Tornillos 4.0x25mm (melamina 15mm)</t>
-  </si>
-  <si>
     <t>609(275x185)</t>
   </si>
   <si>
@@ -583,19 +578,43 @@
     <t>1 Nivel de burbuja (30 cm)</t>
   </si>
   <si>
-    <t>50 Soportes de repisa</t>
-  </si>
-  <si>
     <t>1 broca para madera o metal de 3mm</t>
   </si>
   <si>
     <t>1 bernier o calibrador</t>
   </si>
   <si>
-    <t>1 caution + pomada + estaño</t>
-  </si>
-  <si>
     <t>1 Avellanador con tope de 8mm</t>
+  </si>
+  <si>
+    <t>Preguntar precio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 caution </t>
+  </si>
+  <si>
+    <t>1 pomada + estaño</t>
+  </si>
+  <si>
+    <t>100 Tornillos 4.0x50mm (melamina 18mm)</t>
+  </si>
+  <si>
+    <t>100 Tornillos 4.0x25mm (melamina 18mm)</t>
+  </si>
+  <si>
+    <t>50 Soportes de repisa (ver broca de 4mm)</t>
+  </si>
+  <si>
+    <t>Zapateros</t>
+  </si>
+  <si>
+    <t>Bisagra zapatero metal</t>
+  </si>
+  <si>
+    <t>Bisagra zapatero plastico</t>
+  </si>
+  <si>
+    <t>Broca de 18 mm</t>
   </si>
 </sst>
 </file>
@@ -1553,7 +1572,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC1BAC92-B706-4ADC-AE6C-28D0DABEB4BB}">
-  <dimension ref="A1:I112"/>
+  <dimension ref="A1:I117"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="61.42578125" bestFit="1" customWidth="1"/>
@@ -1583,10 +1602,10 @@
         <v>53</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1612,16 +1631,16 @@
         <v>68</v>
       </c>
       <c r="D3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F3">
         <v>610</v>
       </c>
       <c r="G3" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1632,10 +1651,10 @@
         <v>56</v>
       </c>
       <c r="D4" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G4" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1643,18 +1662,18 @@
         <v>50</v>
       </c>
       <c r="D5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B6" t="s">
+        <v>170</v>
+      </c>
+      <c r="D6" t="s">
         <v>171</v>
-      </c>
-      <c r="B6" t="s">
-        <v>172</v>
-      </c>
-      <c r="D6" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -1711,6 +1730,9 @@
       <c r="A11" t="s">
         <v>63</v>
       </c>
+      <c r="B11" t="s">
+        <v>180</v>
+      </c>
       <c r="F11" t="s">
         <v>64</v>
       </c>
@@ -1723,6 +1745,12 @@
         <v>49</v>
       </c>
       <c r="C12" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E12" s="4" t="s">
         <v>49</v>
       </c>
       <c r="F12" s="4" t="s">
@@ -1780,30 +1808,30 @@
         <v>90</v>
       </c>
       <c r="B18" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C18" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D18" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E18" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F18" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="H18">
         <v>80</v>
       </c>
       <c r="I18" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="H19">
         <v>120</v>
@@ -1814,27 +1842,27 @@
         <v>91</v>
       </c>
       <c r="B20" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C20" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D20" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E20" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F20" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="H20" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -1847,19 +1875,19 @@
         <v>93</v>
       </c>
       <c r="B23" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C23" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D23" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E23" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F23" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="H23">
         <v>60</v>
@@ -1867,7 +1895,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="H24">
         <v>40</v>
@@ -1875,7 +1903,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="H25">
         <v>45</v>
@@ -1886,19 +1914,19 @@
         <v>94</v>
       </c>
       <c r="B26" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C26" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D26" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E26" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F26" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -1906,19 +1934,19 @@
         <v>95</v>
       </c>
       <c r="B27" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C27" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D27" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E27" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F27" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -1926,19 +1954,19 @@
         <v>96</v>
       </c>
       <c r="B28" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C28" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D28" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E28" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F28" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -1948,7 +1976,7 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="H30">
         <v>80</v>
@@ -1956,11 +1984,16 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="12" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="11" t="s">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="11" t="s">
         <v>182</v>
       </c>
     </row>
@@ -1981,19 +2014,19 @@
         <v>98</v>
       </c>
       <c r="B36" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C36" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D36" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E36" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F36" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -2001,20 +2034,20 @@
         <v>99</v>
       </c>
       <c r="C37" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="12" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="H38" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="H39">
         <v>50</v>
@@ -2034,62 +2067,62 @@
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="11" t="s">
-        <v>183</v>
+      <c r="A42" s="12" t="s">
+        <v>179</v>
       </c>
       <c r="B42" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C42" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D42" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E42" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F42" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="H43">
         <v>55</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="11" t="s">
-        <v>142</v>
+      <c r="A44" s="12" t="s">
+        <v>140</v>
       </c>
       <c r="H44">
         <v>115</v>
       </c>
       <c r="I44" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="12" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B45" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C45" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D45" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E45" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F45" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -2125,13 +2158,13 @@
     </row>
     <row r="52" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A52" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H52">
         <v>175</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -2146,7 +2179,7 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="H55">
         <v>395</v>
@@ -2154,18 +2187,18 @@
     </row>
     <row r="56" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="H56">
         <v>490</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="H57">
         <v>40</v>
@@ -2174,13 +2207,13 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="11" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H58">
         <v>270</v>
       </c>
       <c r="I58" s="4" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -2215,10 +2248,10 @@
         <v>88</v>
       </c>
       <c r="H63" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="I63" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -2229,7 +2262,7 @@
         <v>100</v>
       </c>
       <c r="H64" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -2239,21 +2272,21 @@
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="11" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="H66" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="I66" s="13" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="11" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H67" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I67" s="13"/>
     </row>
@@ -2273,19 +2306,19 @@
         <v>109</v>
       </c>
       <c r="B70" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C70" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D70" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E70" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F70" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -2293,19 +2326,19 @@
         <v>110</v>
       </c>
       <c r="B71" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C71" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D71" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E71" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F71" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -2318,19 +2351,19 @@
         <v>112</v>
       </c>
       <c r="B73" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C73" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D73" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E73" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F73" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
@@ -2462,23 +2495,23 @@
         <v>124</v>
       </c>
       <c r="B98" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C98" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D98" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E98" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F98" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A99" s="11" t="s">
+      <c r="A99" s="12" t="s">
         <v>125</v>
       </c>
     </row>
@@ -2497,19 +2530,19 @@
         <v>128</v>
       </c>
       <c r="B102" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C102" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D102" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E102" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F102" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.25">
@@ -2531,33 +2564,33 @@
       </c>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A106" s="11" t="s">
+      <c r="A106" s="12" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A107" s="11" t="s">
+      <c r="A107" s="12" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A108" s="11" t="s">
+      <c r="A108" s="12" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>135</v>
+        <v>183</v>
       </c>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>136</v>
+        <v>184</v>
       </c>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" s="11" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="H111">
         <v>30</v>
@@ -2565,7 +2598,33 @@
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112" s="12" t="s">
-        <v>179</v>
+        <v>185</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A114" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="B114" s="9"/>
+      <c r="C114" s="9"/>
+      <c r="D114" s="9"/>
+      <c r="E114" s="10"/>
+      <c r="F114" s="9"/>
+      <c r="G114" s="9"/>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -2592,7 +2651,7 @@
     </row>
     <row r="44" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G44" s="11" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="45" spans="7:7" x14ac:dyDescent="0.25">
@@ -2602,12 +2661,12 @@
     </row>
     <row r="46" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G46" s="11" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="47" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G47" s="11" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="48" spans="7:7" x14ac:dyDescent="0.25">
@@ -2617,7 +2676,7 @@
     </row>
     <row r="49" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G49" s="11" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="51" spans="7:7" x14ac:dyDescent="0.25">
@@ -2637,7 +2696,7 @@
     </row>
     <row r="54" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G54" s="11" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="55" spans="7:7" x14ac:dyDescent="0.25">
@@ -2647,12 +2706,12 @@
     </row>
     <row r="56" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G56" s="11" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="57" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G57" s="11" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="59" spans="7:7" x14ac:dyDescent="0.25">
@@ -2667,7 +2726,7 @@
     </row>
     <row r="61" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G61" s="11" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="62" spans="7:7" x14ac:dyDescent="0.25">
@@ -2677,17 +2736,17 @@
     </row>
     <row r="63" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G63" s="11" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="64" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G64" s="11" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="65" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G65" s="11" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="67" spans="7:7" x14ac:dyDescent="0.25">
@@ -2717,12 +2776,12 @@
     </row>
     <row r="72" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G72" s="11" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="73" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G73" s="11" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="75" spans="7:7" x14ac:dyDescent="0.25">
@@ -2817,7 +2876,7 @@
     </row>
     <row r="95" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G95" s="11" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
mueble con diagram de corte finalizado
</commit_message>
<xml_diff>
--- a/PROYECTOS/MEZANINE MA/Lista de materiales.xlsx
+++ b/PROYECTOS/MEZANINE MA/Lista de materiales.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30411"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30416"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VIC\Downloads\CURSO SKETCHUP\PROYECTOS\MEZANINE MA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86837F61-14C7-4F70-A68A-0EDD07C36CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E999AAA-93D6-439F-97A8-CE56E2F851FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30612" yWindow="4224" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{9C38CAA7-9F0A-40CC-8992-24B3D9ED1EBA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{9C38CAA7-9F0A-40CC-8992-24B3D9ED1EBA}"/>
   </bookViews>
   <sheets>
     <sheet name="Presupuesto" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="193">
   <si>
     <t>LISTA DE MATERIALES</t>
   </si>
@@ -446,13 +446,7 @@
     <t>100 Tornillos 3.5x15mm (melamina 15mm, bisagras y correderas)</t>
   </si>
   <si>
-    <t>609(275x185)</t>
-  </si>
-  <si>
     <t>810(275x185)</t>
-  </si>
-  <si>
-    <t>719(275x186)</t>
   </si>
   <si>
     <t>365 (marca Total 8v)</t>
@@ -565,9 +559,6 @@
 69252501 Ventas (Hugo Maydana)</t>
   </si>
   <si>
-    <t>667 (275x185x15)</t>
-  </si>
-  <si>
     <t>793 (275x185x18)</t>
   </si>
   <si>
@@ -615,6 +606,25 @@
   </si>
   <si>
     <t>Broca de 18 mm</t>
+  </si>
+  <si>
+    <t>5mm Reborde
+5mm Grosor sierra</t>
+  </si>
+  <si>
+    <t>719(275x186) /Subio a 777</t>
+  </si>
+  <si>
+    <t>609(275x185) /Subio a 660</t>
+  </si>
+  <si>
+    <t>3 (0.6mm)</t>
+  </si>
+  <si>
+    <t>2.5 (0.5mm)</t>
+  </si>
+  <si>
+    <t>667 (275x184x15) / 688</t>
   </si>
 </sst>
 </file>
@@ -1578,7 +1588,7 @@
     <col min="1" max="1" width="38.85546875" customWidth="1"/>
     <col min="2" max="2" width="24.5703125" customWidth="1"/>
     <col min="3" max="3" width="24.140625" customWidth="1"/>
-    <col min="4" max="4" width="23.28515625" customWidth="1"/>
+    <col min="4" max="4" width="26.7109375" customWidth="1"/>
     <col min="5" max="5" width="30.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="23.42578125" customWidth="1"/>
     <col min="8" max="8" width="30.28515625" customWidth="1"/>
@@ -1602,10 +1612,10 @@
         <v>53</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1631,16 +1641,16 @@
         <v>68</v>
       </c>
       <c r="D3" t="s">
-        <v>135</v>
+        <v>189</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="F3">
         <v>610</v>
       </c>
       <c r="G3" t="s">
-        <v>173</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1651,10 +1661,10 @@
         <v>56</v>
       </c>
       <c r="D4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G4" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1662,26 +1672,26 @@
         <v>50</v>
       </c>
       <c r="D5" t="s">
-        <v>137</v>
+        <v>188</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>167</v>
+      </c>
+      <c r="B6" t="s">
+        <v>168</v>
+      </c>
+      <c r="D6" t="s">
         <v>169</v>
-      </c>
-      <c r="B6" t="s">
-        <v>170</v>
-      </c>
-      <c r="D6" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>44</v>
       </c>
-      <c r="B7">
-        <v>3</v>
+      <c r="B7" t="s">
+        <v>190</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>66</v>
@@ -1695,8 +1705,8 @@
       <c r="F7" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="G7" s="4">
-        <v>2.5</v>
+      <c r="G7" s="4" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1731,7 +1741,7 @@
         <v>63</v>
       </c>
       <c r="B11" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="F11" t="s">
         <v>64</v>
@@ -1748,7 +1758,7 @@
         <v>49</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>49</v>
+        <v>187</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>49</v>
@@ -1808,30 +1818,30 @@
         <v>90</v>
       </c>
       <c r="B18" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C18" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D18" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E18" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F18" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="H18">
         <v>80</v>
       </c>
       <c r="I18" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H19">
         <v>120</v>
@@ -1842,27 +1852,27 @@
         <v>91</v>
       </c>
       <c r="B20" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C20" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D20" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E20" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F20" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="H20" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -1875,19 +1885,19 @@
         <v>93</v>
       </c>
       <c r="B23" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C23" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D23" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E23" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F23" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="H23">
         <v>60</v>
@@ -1895,7 +1905,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="H24">
         <v>40</v>
@@ -1903,7 +1913,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="H25">
         <v>45</v>
@@ -1914,19 +1924,19 @@
         <v>94</v>
       </c>
       <c r="B26" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C26" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D26" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E26" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F26" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -1934,19 +1944,19 @@
         <v>95</v>
       </c>
       <c r="B27" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C27" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D27" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E27" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F27" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -1954,19 +1964,19 @@
         <v>96</v>
       </c>
       <c r="B28" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C28" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D28" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E28" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F28" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -1976,7 +1986,7 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="H30">
         <v>80</v>
@@ -1984,17 +1994,17 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -2014,19 +2024,19 @@
         <v>98</v>
       </c>
       <c r="B36" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C36" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D36" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E36" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F36" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -2034,20 +2044,20 @@
         <v>99</v>
       </c>
       <c r="C37" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="12" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="H38" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H39">
         <v>50</v>
@@ -2068,27 +2078,27 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="12" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="B42" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C42" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D42" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E42" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F42" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="H43">
         <v>55</v>
@@ -2096,33 +2106,33 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="12" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="H44">
         <v>115</v>
       </c>
       <c r="I44" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="12" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B45" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C45" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D45" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E45" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F45" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -2158,13 +2168,13 @@
     </row>
     <row r="52" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A52" s="12" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="H52">
         <v>175</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -2179,7 +2189,7 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="H55">
         <v>395</v>
@@ -2187,18 +2197,18 @@
     </row>
     <row r="56" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="H56">
         <v>490</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="H57">
         <v>40</v>
@@ -2207,13 +2217,13 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="11" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="H58">
         <v>270</v>
       </c>
       <c r="I58" s="4" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -2248,10 +2258,10 @@
         <v>88</v>
       </c>
       <c r="H63" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I63" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -2262,7 +2272,7 @@
         <v>100</v>
       </c>
       <c r="H64" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -2272,21 +2282,21 @@
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="11" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="H66" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="I66" s="13" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="11" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="H67" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="I67" s="13"/>
     </row>
@@ -2306,19 +2316,19 @@
         <v>109</v>
       </c>
       <c r="B70" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C70" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D70" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E70" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F70" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
@@ -2326,19 +2336,19 @@
         <v>110</v>
       </c>
       <c r="B71" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C71" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D71" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E71" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F71" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
@@ -2351,19 +2361,19 @@
         <v>112</v>
       </c>
       <c r="B73" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C73" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D73" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E73" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F73" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
@@ -2495,19 +2505,19 @@
         <v>124</v>
       </c>
       <c r="B98" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C98" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D98" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E98" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F98" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.25">
@@ -2530,19 +2540,19 @@
         <v>128</v>
       </c>
       <c r="B102" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C102" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D102" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E102" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F102" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.25">
@@ -2580,17 +2590,17 @@
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" s="11" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H111">
         <v>30</v>
@@ -2598,12 +2608,12 @@
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112" s="12" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" s="8" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="B114" s="9"/>
       <c r="C114" s="9"/>
@@ -2614,17 +2624,17 @@
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -2651,7 +2661,7 @@
     </row>
     <row r="44" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G44" s="11" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="45" spans="7:7" x14ac:dyDescent="0.25">
@@ -2661,12 +2671,12 @@
     </row>
     <row r="46" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G46" s="11" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="47" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G47" s="11" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="48" spans="7:7" x14ac:dyDescent="0.25">
@@ -2676,7 +2686,7 @@
     </row>
     <row r="49" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G49" s="11" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="51" spans="7:7" x14ac:dyDescent="0.25">
@@ -2696,7 +2706,7 @@
     </row>
     <row r="54" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G54" s="11" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="55" spans="7:7" x14ac:dyDescent="0.25">
@@ -2706,12 +2716,12 @@
     </row>
     <row r="56" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G56" s="11" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="57" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G57" s="11" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="59" spans="7:7" x14ac:dyDescent="0.25">
@@ -2726,7 +2736,7 @@
     </row>
     <row r="61" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G61" s="11" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="62" spans="7:7" x14ac:dyDescent="0.25">
@@ -2736,17 +2746,17 @@
     </row>
     <row r="63" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G63" s="11" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="64" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G64" s="11" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="65" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G65" s="11" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="67" spans="7:7" x14ac:dyDescent="0.25">
@@ -2776,12 +2786,12 @@
     </row>
     <row r="72" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G72" s="11" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="73" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G73" s="11" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="75" spans="7:7" x14ac:dyDescent="0.25">
@@ -2876,7 +2886,7 @@
     </row>
     <row r="95" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G95" s="11" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>